<commit_message>
Gate 3: order totals - every per-unit number multiplied by the set count
Van: "what if we add amount as well? like sets, and everything will be counted
with formula?" So: one input (sets in this order, default 300) and a second
tile row that turns the unit economics into order money - goods with the 30/70
deposit/balance split shown inline, landed total, the import-VAT out-and-back,
contribution if every set sells, and the same after the profit-tax reserve.

Workbook first: Sheet 3 rows 43-51 carry identical formulas, rebuilt and
recalculated in Excel; the section header says where the real order plan lives
(Sheets 6 + 8), because a quick-multiplication row is not a demand model - it
answers "how much money does this order touch", not "how many will sell".

Suite 265/265: the five order tiles assert against the mirror AND against the
workbook's freshly recalculated cells C45/C48/C49/C50/C51 as literals.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workbook/amazon-de-seller-workbook-v4-EN.xlsx
+++ b/workbook/amazon-de-seller-workbook-v4-EN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/van/Desktop/Helium Analysis/ANALYST/easestore-tools/workbook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47796580-4321-C34D-94B2-209F9E2701EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27273E16-F697-4343-BD00-534328004F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -398,7 +398,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="519">
   <si>
     <t>Amazon.de Seller Workbook — v4</t>
   </si>
@@ -965,6 +965,36 @@
   </si>
   <si>
     <t>Cross-check the FBA fee against real dimensions: €4.55 is not a 12 cm box. H10 exports sometimes mislabel inches as cm.</t>
+  </si>
+  <si>
+    <t>Order totals — quick math (the real order plan lives in Sheets 6 + 8)</t>
+  </si>
+  <si>
+    <t>Sets in this order</t>
+  </si>
+  <si>
+    <t>Goods (EXW × sets)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   deposit 30% at order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   balance 70% after passed inspection</t>
+  </si>
+  <si>
+    <t>Landed total (cash into stock)</t>
+  </si>
+  <si>
+    <t>Import VAT at customs (out, then back)</t>
+  </si>
+  <si>
+    <t>Paid at Hamburg, recovered through the German VAT return roughly two months later - the cash hole Gate 5 draws.</t>
+  </si>
+  <si>
+    <t>Contribution if ALL sets sell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   after profit-tax reserve</t>
   </si>
   <si>
     <t>Selection checklist. Any NO in block A is an automatic reject.</t>
@@ -2657,12 +2687,12 @@
     </row>
     <row r="2" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>379</v>
+        <v>389</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="210" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.2">
@@ -2673,7 +2703,7 @@
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B6" s="11" t="s">
-        <v>381</v>
+        <v>391</v>
       </c>
       <c r="C6" s="34">
         <f>'6 Order size'!C24</f>
@@ -2691,7 +2721,7 @@
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B8" s="11" t="s">
-        <v>382</v>
+        <v>392</v>
       </c>
       <c r="C8" s="27">
         <f>IFERROR(C6*C7,"")</f>
@@ -2700,7 +2730,7 @@
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B9" s="11" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
       <c r="C9" s="26">
         <v>0.3</v>
@@ -2708,7 +2738,7 @@
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B10" s="11" t="s">
-        <v>384</v>
+        <v>394</v>
       </c>
       <c r="C10" s="22">
         <v>2</v>
@@ -2716,7 +2746,7 @@
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B11" s="11" t="s">
-        <v>385</v>
+        <v>395</v>
       </c>
       <c r="C11" s="22">
         <v>3</v>
@@ -2724,7 +2754,7 @@
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B12" s="11" t="s">
-        <v>386</v>
+        <v>396</v>
       </c>
       <c r="C12" s="27">
         <f>IFERROR(ROUND(0.19*C8,0),"")</f>
@@ -2733,7 +2763,7 @@
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B13" s="11" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="C13" s="22">
         <v>2</v>
@@ -2741,7 +2771,7 @@
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B14" s="11" t="s">
-        <v>388</v>
+        <v>398</v>
       </c>
       <c r="C14" s="33">
         <f>'3 Unit economics'!C26</f>
@@ -2750,7 +2780,7 @@
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B15" s="11" t="s">
-        <v>389</v>
+        <v>399</v>
       </c>
       <c r="C15" s="25">
         <v>6500</v>
@@ -2761,22 +2791,22 @@
         <v>68</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>390</v>
+        <v>400</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>391</v>
+        <v>401</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>392</v>
+        <v>402</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>393</v>
+        <v>403</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>394</v>
+        <v>404</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="26" x14ac:dyDescent="0.2">
@@ -2806,7 +2836,7 @@
         <v>5003</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>396</v>
+        <v>406</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.2">
@@ -2890,7 +2920,7 @@
         <v>1887</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>397</v>
+        <v>407</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.2">
@@ -3138,7 +3168,7 @@
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B32" s="5" t="s">
-        <v>398</v>
+        <v>408</v>
       </c>
       <c r="C32" s="17">
         <f>MIN(H17:H29)</f>
@@ -3153,12 +3183,12 @@
     </row>
     <row r="35" spans="2:3" ht="272" x14ac:dyDescent="0.2">
       <c r="B35" s="3" t="s">
-        <v>399</v>
+        <v>409</v>
       </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B37" s="5" t="s">
-        <v>400</v>
+        <v>410</v>
       </c>
       <c r="C37" s="23">
         <f>'2 Order timing'!C18+45+14</f>
@@ -3167,7 +3197,7 @@
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B38" s="5" t="s">
-        <v>401</v>
+        <v>411</v>
       </c>
       <c r="C38" s="30">
         <f>IFERROR(ROUND(365/C37,1),"")</f>
@@ -3208,12 +3238,12 @@
     </row>
     <row r="2" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>402</v>
+        <v>412</v>
       </c>
     </row>
     <row r="3" spans="2:13" ht="358" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>403</v>
+        <v>413</v>
       </c>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.2">
@@ -3221,37 +3251,37 @@
         <v>68</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>404</v>
+        <v>414</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>405</v>
+        <v>415</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>406</v>
+        <v>416</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>407</v>
+        <v>417</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>408</v>
+        <v>418</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>409</v>
+        <v>419</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>410</v>
+        <v>420</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>411</v>
+        <v>421</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>412</v>
+        <v>422</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>413</v>
+        <v>423</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>414</v>
+        <v>424</v>
       </c>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.2">
@@ -3689,12 +3719,12 @@
     </row>
     <row r="20" spans="2:13" ht="260" x14ac:dyDescent="0.2">
       <c r="B20" s="3" t="s">
-        <v>415</v>
+        <v>425</v>
       </c>
     </row>
     <row r="21" spans="2:13" ht="247" x14ac:dyDescent="0.2">
       <c r="B21" s="3" t="s">
-        <v>416</v>
+        <v>426</v>
       </c>
     </row>
   </sheetData>
@@ -3728,17 +3758,17 @@
     </row>
     <row r="2" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="224" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>418</v>
+        <v>428</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="C5" s="23">
         <f>COUNTIF($F$12:$F$61,"NOT REIMBURSED — check &amp; claim")</f>
@@ -3747,24 +3777,24 @@
     </row>
     <row r="7" spans="2:6" ht="156" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
-        <v>420</v>
+        <v>430</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B11" s="4" t="s">
-        <v>421</v>
+        <v>431</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>422</v>
+        <v>432</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>423</v>
+        <v>433</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>424</v>
+        <v>434</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>425</v>
+        <v>435</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.2">
@@ -3772,10 +3802,10 @@
         <v>46206</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>426</v>
+        <v>436</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>427</v>
+        <v>437</v>
       </c>
       <c r="E12" s="22">
         <v>2</v>
@@ -3790,10 +3820,10 @@
         <v>46222</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>428</v>
+        <v>438</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>429</v>
+        <v>439</v>
       </c>
       <c r="E13" s="22">
         <v>1</v>
@@ -4285,18 +4315,18 @@
     </row>
     <row r="64" spans="2:6" ht="117" x14ac:dyDescent="0.2">
       <c r="B64" s="3" t="s">
-        <v>430</v>
+        <v>440</v>
       </c>
     </row>
     <row r="67" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B67" s="4" t="s">
-        <v>421</v>
+        <v>431</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>422</v>
+        <v>432</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>431</v>
+        <v>441</v>
       </c>
     </row>
     <row r="68" spans="2:4" x14ac:dyDescent="0.2">
@@ -4304,7 +4334,7 @@
         <v>46224</v>
       </c>
       <c r="C68" s="9" t="s">
-        <v>426</v>
+        <v>436</v>
       </c>
       <c r="D68" s="25">
         <v>18.399999999999999</v>
@@ -4557,12 +4587,12 @@
     </row>
     <row r="120" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B120" s="4" t="s">
-        <v>432</v>
+        <v>442</v>
       </c>
     </row>
     <row r="121" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B121" s="11" t="s">
-        <v>433</v>
+        <v>443</v>
       </c>
       <c r="C121" s="35">
         <v>25</v>
@@ -4570,7 +4600,7 @@
     </row>
     <row r="122" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B122" s="11" t="s">
-        <v>434</v>
+        <v>444</v>
       </c>
       <c r="C122" s="35">
         <v>18</v>
@@ -4578,7 +4608,7 @@
     </row>
     <row r="123" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B123" s="11" t="s">
-        <v>435</v>
+        <v>445</v>
       </c>
       <c r="C123" s="35">
         <v>4</v>
@@ -4586,7 +4616,7 @@
     </row>
     <row r="124" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B124" s="11" t="s">
-        <v>436</v>
+        <v>446</v>
       </c>
       <c r="C124" s="22">
         <v>350</v>
@@ -4594,7 +4624,7 @@
     </row>
     <row r="125" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B125" s="11" t="s">
-        <v>437</v>
+        <v>447</v>
       </c>
       <c r="C125" s="25">
         <v>4.55</v>
@@ -4602,7 +4632,7 @@
     </row>
     <row r="126" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B126" s="11" t="s">
-        <v>438</v>
+        <v>448</v>
       </c>
       <c r="C126" s="14">
         <f>ROUND(C121*C122*C123/1000,2)</f>
@@ -4611,7 +4641,7 @@
     </row>
     <row r="127" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B127" s="11" t="s">
-        <v>439</v>
+        <v>449</v>
       </c>
       <c r="C127" s="29">
         <f>MAX(C121:C123)</f>
@@ -4620,55 +4650,55 @@
     </row>
     <row r="129" spans="2:3" ht="247" x14ac:dyDescent="0.2">
       <c r="B129" s="3" t="s">
-        <v>440</v>
+        <v>450</v>
       </c>
     </row>
     <row r="131" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B131" s="4" t="s">
-        <v>441</v>
+        <v>451</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>442</v>
+        <v>452</v>
       </c>
     </row>
     <row r="132" spans="2:3" ht="56" x14ac:dyDescent="0.2">
       <c r="B132" s="2" t="s">
-        <v>443</v>
+        <v>453</v>
       </c>
       <c r="C132" s="9" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="133" spans="2:3" ht="42" x14ac:dyDescent="0.2">
       <c r="B133" s="2" t="s">
-        <v>444</v>
+        <v>454</v>
       </c>
       <c r="C133" s="9" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="134" spans="2:3" ht="42" x14ac:dyDescent="0.2">
       <c r="B134" s="2" t="s">
-        <v>445</v>
+        <v>455</v>
       </c>
       <c r="C134" s="9" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="135" spans="2:3" ht="70" x14ac:dyDescent="0.2">
       <c r="B135" s="2" t="s">
-        <v>446</v>
+        <v>456</v>
       </c>
       <c r="C135" s="9" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="136" spans="2:3" ht="56" x14ac:dyDescent="0.2">
       <c r="B136" s="2" t="s">
-        <v>447</v>
+        <v>457</v>
       </c>
       <c r="C136" s="9" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -4700,36 +4730,36 @@
     </row>
     <row r="2" spans="2:4" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="70" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B5" s="11" t="s">
-        <v>450</v>
+        <v>460</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>451</v>
+        <v>461</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" s="4" t="s">
-        <v>452</v>
+        <v>462</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>453</v>
+        <v>463</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>454</v>
+        <v>464</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B8" s="9" t="s">
-        <v>455</v>
+        <v>465</v>
       </c>
       <c r="C8" s="22">
         <v>46</v>
@@ -4741,7 +4771,7 @@
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B9" s="9" t="s">
-        <v>456</v>
+        <v>466</v>
       </c>
       <c r="C9" s="22">
         <v>21</v>
@@ -4753,7 +4783,7 @@
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B10" s="9" t="s">
-        <v>457</v>
+        <v>467</v>
       </c>
       <c r="C10" s="22">
         <v>18</v>
@@ -4765,7 +4795,7 @@
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B11" s="9" t="s">
-        <v>458</v>
+        <v>468</v>
       </c>
       <c r="C11" s="22">
         <v>15</v>
@@ -4777,7 +4807,7 @@
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B12" s="9" t="s">
-        <v>459</v>
+        <v>469</v>
       </c>
       <c r="C12" s="22">
         <v>8</v>
@@ -4829,7 +4859,7 @@
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B19" s="5" t="s">
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="C19" s="5" t="str">
         <f>IFERROR(INDEX(B8:B17,MATCH(MAX(C8:C17),C8:C17,0)),"—")</f>
@@ -4838,7 +4868,7 @@
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B20" s="5" t="s">
-        <v>461</v>
+        <v>471</v>
       </c>
       <c r="C20" s="18">
         <f>IFERROR(MAX(C8:C17)/SUM(C8:C17),"")</f>
@@ -4856,61 +4886,61 @@
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B23" s="4" t="s">
-        <v>462</v>
+        <v>472</v>
       </c>
       <c r="C23" s="4"/>
     </row>
     <row r="24" spans="2:4" ht="28" x14ac:dyDescent="0.2">
       <c r="B24" s="2" t="s">
-        <v>463</v>
+        <v>473</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="28" x14ac:dyDescent="0.2">
       <c r="B25" s="2" t="s">
-        <v>464</v>
+        <v>474</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="28" x14ac:dyDescent="0.2">
       <c r="B26" s="2" t="s">
-        <v>465</v>
+        <v>475</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B27" s="2" t="s">
-        <v>466</v>
+        <v>476</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="28" spans="2:4" ht="28" x14ac:dyDescent="0.2">
       <c r="B28" s="2" t="s">
-        <v>467</v>
+        <v>477</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="29" spans="2:4" ht="28" x14ac:dyDescent="0.2">
       <c r="B29" s="2" t="s">
-        <v>468</v>
+        <v>478</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B30" s="5" t="s">
-        <v>469</v>
+        <v>479</v>
       </c>
       <c r="C30" s="23">
         <f>COUNTIF(C24:C29,"YES")</f>
@@ -4928,7 +4958,7 @@
     </row>
     <row r="33" spans="2:2" ht="39" x14ac:dyDescent="0.2">
       <c r="B33" s="3" t="s">
-        <v>470</v>
+        <v>480</v>
       </c>
     </row>
   </sheetData>
@@ -4958,23 +4988,23 @@
     </row>
     <row r="2" spans="2:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>471</v>
+        <v>481</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="70" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>472</v>
+        <v>482</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B5" s="4" t="s">
-        <v>473</v>
+        <v>483</v>
       </c>
       <c r="C5" s="4"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B6" s="11" t="s">
-        <v>474</v>
+        <v>484</v>
       </c>
       <c r="C6" s="34">
         <f>'8 Cash flow'!C15</f>
@@ -4983,18 +5013,18 @@
     </row>
     <row r="7" spans="2:6" ht="117" x14ac:dyDescent="0.2">
       <c r="B7" s="11" t="s">
-        <v>475</v>
+        <v>485</v>
       </c>
       <c r="C7" s="12">
         <v>400</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>476</v>
+        <v>486</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B8" s="11" t="s">
-        <v>477</v>
+        <v>487</v>
       </c>
       <c r="C8" s="26">
         <v>0.4</v>
@@ -5002,21 +5032,21 @@
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B10" s="4" t="s">
-        <v>478</v>
+        <v>488</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>479</v>
+        <v>489</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>481</v>
+        <v>491</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B11" s="11" t="s">
-        <v>482</v>
+        <v>492</v>
       </c>
       <c r="C11" s="22">
         <v>1</v>
@@ -5028,7 +5058,7 @@
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B12" s="11" t="s">
-        <v>483</v>
+        <v>493</v>
       </c>
       <c r="C12" s="12">
         <v>300</v>
@@ -5040,7 +5070,7 @@
     </row>
     <row r="13" spans="2:6" ht="182" x14ac:dyDescent="0.2">
       <c r="B13" s="11" t="s">
-        <v>484</v>
+        <v>494</v>
       </c>
       <c r="C13" s="33">
         <f>'3 Unit economics'!C26+'3 Unit economics'!C28</f>
@@ -5051,12 +5081,12 @@
       </c>
       <c r="E13" s="25"/>
       <c r="F13" s="3" t="s">
-        <v>485</v>
+        <v>495</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B14" s="11" t="s">
-        <v>486</v>
+        <v>496</v>
       </c>
       <c r="C14" s="33">
         <f>'6 Order size'!C15</f>
@@ -5069,7 +5099,7 @@
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B15" s="11" t="s">
-        <v>487</v>
+        <v>497</v>
       </c>
       <c r="C15" s="12">
         <v>6000</v>
@@ -5081,7 +5111,7 @@
     </row>
     <row r="16" spans="2:6" ht="91" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
-        <v>488</v>
+        <v>498</v>
       </c>
       <c r="C16" s="25">
         <v>3</v>
@@ -5091,23 +5121,23 @@
       </c>
       <c r="E16" s="25"/>
       <c r="F16" s="3" t="s">
-        <v>489</v>
+        <v>499</v>
       </c>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.2">
       <c r="C18" s="5" t="s">
-        <v>490</v>
+        <v>500</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>491</v>
+        <v>501</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>492</v>
+        <v>502</v>
       </c>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B19" s="4" t="s">
-        <v>493</v>
+        <v>503</v>
       </c>
       <c r="C19" s="36">
         <v>1</v>
@@ -5148,7 +5178,7 @@
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B20" s="11" t="s">
-        <v>494</v>
+        <v>504</v>
       </c>
       <c r="C20" s="13">
         <f t="shared" ref="C20:N20" si="0">IF(OR($C$11="",C$19&lt;$C$11),0,ROUND($C$12*IF(C$19-$C$11=0,$C$8,IF(C$19-$C$11=1,($C$8+1)/2,1)),0))</f>
@@ -5201,7 +5231,7 @@
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B21" s="11" t="s">
-        <v>495</v>
+        <v>505</v>
       </c>
       <c r="C21" s="13">
         <f t="shared" ref="C21:N21" si="1">IF(OR($D$11="",C$19&lt;$D$11),0,ROUND($D$12*IF(C$19-$D$11=0,$C$8,IF(C$19-$D$11=1,($C$8+1)/2,1)),0))</f>
@@ -5254,7 +5284,7 @@
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B22" s="11" t="s">
-        <v>496</v>
+        <v>506</v>
       </c>
       <c r="C22" s="13">
         <f t="shared" ref="C22:N22" si="2">IF(OR($E$11="",C$19&lt;$E$11),0,ROUND($E$12*IF(C$19-$E$11=0,$C$8,IF(C$19-$E$11=1,($C$8+1)/2,1)),0))</f>
@@ -5307,7 +5337,7 @@
     </row>
     <row r="24" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B24" s="11" t="s">
-        <v>497</v>
+        <v>507</v>
       </c>
       <c r="C24" s="13">
         <f t="shared" ref="C24:N24" si="3">ROUND(C20*N($C$13)+C21*N($D$13)+C22*N($E$13),0)</f>
@@ -5360,7 +5390,7 @@
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B25" s="11" t="s">
-        <v>498</v>
+        <v>508</v>
       </c>
       <c r="C25" s="13">
         <f t="shared" ref="C25:M25" si="4">ROUND(IF(OR($C$11="",D$19=$C$11),0,D20)*N($C$14)+IF(OR($D$11="",D$19=$D$11),0,D21)*N($D$14)+IF(OR($E$11="",D$19=$E$11),0,D22)*N($E$14),0)</f>
@@ -5413,7 +5443,7 @@
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B26" s="11" t="s">
-        <v>499</v>
+        <v>509</v>
       </c>
       <c r="C26" s="13">
         <f t="shared" ref="C26:N26" si="5">SUMPRODUCT(($C$11:$E$11=C$19+1)*$C$15:$E$15)+IF(C$19=1,SUMPRODUCT(($C$11:$E$11=1)*$C$15:$E$15),0)</f>
@@ -5466,7 +5496,7 @@
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B27" s="11" t="s">
-        <v>500</v>
+        <v>510</v>
       </c>
       <c r="C27" s="13">
         <f t="shared" ref="C27:N27" si="6">ROUND(C20*N($C$16)+C21*N($D$16)+C22*N($E$16),0)</f>
@@ -5519,7 +5549,7 @@
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B28" s="11" t="s">
-        <v>501</v>
+        <v>511</v>
       </c>
       <c r="C28" s="13">
         <f t="shared" ref="C28:N28" si="7">$C$7</f>
@@ -5572,7 +5602,7 @@
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B29" s="5" t="s">
-        <v>502</v>
+        <v>512</v>
       </c>
       <c r="C29" s="17">
         <f t="shared" ref="C29:N29" si="8">C24-C25-C26-C27-C28</f>
@@ -5625,7 +5655,7 @@
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B30" s="5" t="s">
-        <v>503</v>
+        <v>513</v>
       </c>
       <c r="C30" s="17">
         <f>$C$6+C29</f>
@@ -5678,7 +5708,7 @@
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B32" s="5" t="s">
-        <v>504</v>
+        <v>514</v>
       </c>
       <c r="C32" s="17">
         <f>MIN(C30:N30)</f>
@@ -5693,7 +5723,7 @@
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B34" s="11" t="s">
-        <v>505</v>
+        <v>515</v>
       </c>
       <c r="C34" s="13">
         <f>SUM(C29:F29)</f>
@@ -5710,17 +5740,17 @@
     </row>
     <row r="36" spans="2:11" ht="65" x14ac:dyDescent="0.2">
       <c r="B36" s="3" t="s">
-        <v>506</v>
+        <v>516</v>
       </c>
     </row>
     <row r="37" spans="2:11" ht="78" x14ac:dyDescent="0.2">
       <c r="B37" s="3" t="s">
-        <v>507</v>
+        <v>517</v>
       </c>
     </row>
     <row r="38" spans="2:11" ht="52" x14ac:dyDescent="0.2">
       <c r="B38" s="3" t="s">
-        <v>508</v>
+        <v>518</v>
       </c>
     </row>
   </sheetData>
@@ -6619,7 +6649,7 @@
   <sheetPr>
     <tabColor rgb="FF4472C4"/>
   </sheetPr>
-  <dimension ref="B1:E41"/>
+  <dimension ref="B1:E51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -6990,6 +7020,86 @@
     <row r="41" spans="2:5" ht="26" x14ac:dyDescent="0.2">
       <c r="B41" s="3" t="s">
         <v>188</v>
+      </c>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B43" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="C43" s="4"/>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B44" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="C44" s="22">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B45" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="C45" s="27">
+        <f>C14*C44</f>
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B46" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="C46" s="27">
+        <f>0.3*C45</f>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B47" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="C47" s="27">
+        <f>0.7*C45</f>
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B48" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="C48" s="27">
+        <f>-C27*C44</f>
+        <v>3878.8199999999997</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" ht="26" x14ac:dyDescent="0.2">
+      <c r="B49" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="C49" s="27">
+        <f>0.19*(C14+C15)*(1+C16)*C44</f>
+        <v>714.17579999999987</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B50" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="C50" s="28">
+        <f>C29*C44</f>
+        <v>6101.8711764705904</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B51" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="C51" s="27">
+        <f>C35*C44</f>
+        <v>4271.3098235294128</v>
       </c>
     </row>
   </sheetData>
@@ -7021,269 +7131,269 @@
     </row>
     <row r="2" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B4" s="4" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B5" s="2" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B7" s="2" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B9" s="2" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B10" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>193</v>
-      </c>
       <c r="E10" s="3" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="26" x14ac:dyDescent="0.2">
       <c r="B11" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B12" s="2" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B13" s="2" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B15" s="4" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B16" s="2" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B17" s="2" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B18" s="2" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B19" s="2" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B20" s="2" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B21" s="2" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B22" s="2" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B23" s="2" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B25" s="4" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B26" s="2" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B27" s="2" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B28" s="2" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B29" s="2" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B30" s="2" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B32" s="5" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="C32" s="5" t="str">
         <f>IF(COUNTIF(C5:C13,"YES")=9,"CLEAN","REJECT")</f>
@@ -7292,7 +7402,7 @@
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B33" s="5" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="C33" s="5" t="str">
         <f>COUNTIF(C16:C23,"YES")&amp;" / 8"</f>
@@ -7301,7 +7411,7 @@
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B34" s="5" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="C34" s="5" t="str">
         <f>COUNTIF(C26:C30,"YES")&amp;" / 5"</f>
@@ -7310,29 +7420,29 @@
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B36" s="3" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B38" s="4" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C38" s="4"/>
     </row>
     <row r="39" spans="2:5" ht="26" x14ac:dyDescent="0.2">
       <c r="B39" s="11" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="C39" s="22">
         <v>75</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B40" s="11" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="C40" s="22">
         <v>300</v>
@@ -7340,18 +7450,18 @@
     </row>
     <row r="41" spans="2:5" ht="26" x14ac:dyDescent="0.2">
       <c r="B41" s="11" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="C41" s="26">
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B42" s="11" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="C42" s="29">
         <f>IFERROR(C40*C41,"")</f>
@@ -7360,7 +7470,7 @@
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B43" s="5" t="s">
-        <v>247</v>
+        <v>257</v>
       </c>
       <c r="C43" s="30">
         <f>IFERROR(C39/C42,"")</f>
@@ -7375,7 +7485,7 @@
     </row>
     <row r="46" spans="2:5" ht="78" x14ac:dyDescent="0.2">
       <c r="B46" s="3" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -7405,17 +7515,17 @@
     </row>
     <row r="2" spans="2:11" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="2:11" ht="42" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B4" s="11" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="C4" s="25">
         <v>6500</v>
@@ -7426,39 +7536,39 @@
         <v>134</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>254</v>
+        <v>264</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>61</v>
@@ -7473,10 +7583,10 @@
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B7" s="2" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="D7" s="12">
         <v>23500</v>
@@ -7491,10 +7601,10 @@
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="D8" s="12">
         <v>95000</v>
@@ -7509,10 +7619,10 @@
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B9" s="2" t="s">
-        <v>267</v>
+        <v>277</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="D9" s="26">
         <v>0.28000000000000003</v>
@@ -7527,10 +7637,10 @@
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B10" s="2" t="s">
-        <v>268</v>
+        <v>278</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="D10" s="22">
         <v>5</v>
@@ -7545,10 +7655,10 @@
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B11" s="2" t="s">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="D11" s="22">
         <v>2</v>
@@ -7563,10 +7673,10 @@
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B12" s="2" t="s">
-        <v>271</v>
+        <v>281</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="D12" s="22">
         <v>1</v>
@@ -7581,10 +7691,10 @@
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B13" s="2" t="s">
-        <v>272</v>
+        <v>282</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="D13" s="26">
         <v>0.55000000000000004</v>
@@ -7599,10 +7709,10 @@
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B14" s="2" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="D14" s="31">
         <v>5.15</v>
@@ -7617,10 +7727,10 @@
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B15" s="2" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="D15" s="26">
         <v>0.54</v>
@@ -7635,10 +7745,10 @@
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B16" s="2" t="s">
-        <v>276</v>
+        <v>286</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="D16" s="26">
         <v>0.4</v>
@@ -7653,10 +7763,10 @@
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B17" s="2" t="s">
-        <v>278</v>
+        <v>288</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>279</v>
+        <v>289</v>
       </c>
       <c r="D17" s="12">
         <v>9000</v>
@@ -7671,13 +7781,13 @@
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B18" s="2" t="s">
-        <v>280</v>
+        <v>290</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>281</v>
+        <v>291</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
@@ -7689,10 +7799,10 @@
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B20" s="4" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
@@ -7705,7 +7815,7 @@
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B21" s="11" t="s">
-        <v>285</v>
+        <v>295</v>
       </c>
       <c r="C21" s="32">
         <v>0.15</v>
@@ -7745,7 +7855,7 @@
     </row>
     <row r="22" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B22" s="11" t="s">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="C22" s="32">
         <v>0.1</v>
@@ -7785,7 +7895,7 @@
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B23" s="11" t="s">
-        <v>287</v>
+        <v>297</v>
       </c>
       <c r="C23" s="32">
         <v>0.1</v>
@@ -7825,7 +7935,7 @@
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B24" s="11" t="s">
-        <v>288</v>
+        <v>298</v>
       </c>
       <c r="C24" s="32">
         <v>0.1</v>
@@ -7865,7 +7975,7 @@
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B25" s="11" t="s">
-        <v>289</v>
+        <v>299</v>
       </c>
       <c r="C25" s="32">
         <v>0.1</v>
@@ -7905,7 +8015,7 @@
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B26" s="11" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="C26" s="32">
         <v>0.05</v>
@@ -7945,7 +8055,7 @@
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B27" s="11" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="C27" s="32">
         <v>0.15</v>
@@ -7985,7 +8095,7 @@
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B28" s="11" t="s">
-        <v>291</v>
+        <v>301</v>
       </c>
       <c r="C28" s="32">
         <v>0.05</v>
@@ -8025,7 +8135,7 @@
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B29" s="11" t="s">
-        <v>292</v>
+        <v>302</v>
       </c>
       <c r="C29" s="32">
         <v>0.15</v>
@@ -8065,7 +8175,7 @@
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B30" s="11" t="s">
-        <v>293</v>
+        <v>303</v>
       </c>
       <c r="C30" s="32">
         <v>0.05</v>
@@ -8105,7 +8215,7 @@
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B32" s="5" t="s">
-        <v>294</v>
+        <v>304</v>
       </c>
       <c r="D32" s="23">
         <f t="shared" ref="D32:K32" si="10">IF(COUNT(D21:D30)&lt;10,"",ROUND(SUMPRODUCT($C$21:$C$30,D21:D30)/2*100,0))</f>
@@ -8142,7 +8252,7 @@
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B33" s="5" t="s">
-        <v>295</v>
+        <v>305</v>
       </c>
       <c r="D33" s="5" t="str">
         <f t="shared" ref="D33:K33" si="11">IF(D18="NO","DISQUALIFIED: compliance",IF(D14="","—",IF(D14&gt;=4,"DISQUALIFIED: single-season","OK")))</f>
@@ -8216,12 +8326,12 @@
     </row>
     <row r="36" spans="2:11" ht="26" x14ac:dyDescent="0.2">
       <c r="B36" s="3" t="s">
-        <v>296</v>
+        <v>306</v>
       </c>
     </row>
     <row r="37" spans="2:11" ht="39" x14ac:dyDescent="0.2">
       <c r="B37" s="3" t="s">
-        <v>297</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>
@@ -8252,12 +8362,12 @@
     </row>
     <row r="2" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="56" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>299</v>
+        <v>309</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.2">
@@ -8268,79 +8378,79 @@
     </row>
     <row r="6" spans="2:5" ht="26" x14ac:dyDescent="0.2">
       <c r="B6" s="11" t="s">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="C6" s="12">
         <v>600</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>301</v>
+        <v>311</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B7" s="11" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="C7" s="12">
         <v>1400</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>303</v>
+        <v>313</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B8" s="11" t="s">
-        <v>304</v>
+        <v>314</v>
       </c>
       <c r="C8" s="25">
         <v>5</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>305</v>
+        <v>315</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B9" s="11" t="s">
-        <v>306</v>
+        <v>316</v>
       </c>
       <c r="C9" s="25">
         <v>1</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>307</v>
+        <v>317</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B10" s="11" t="s">
-        <v>308</v>
+        <v>318</v>
       </c>
       <c r="C10" s="12">
         <v>300</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>309</v>
+        <v>319</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B11" s="11" t="s">
-        <v>310</v>
+        <v>320</v>
       </c>
       <c r="C11" s="25">
         <v>5000</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>311</v>
+        <v>321</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B13" s="4" t="s">
-        <v>312</v>
+        <v>322</v>
       </c>
       <c r="C13" s="4"/>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B14" s="11" t="s">
-        <v>313</v>
+        <v>323</v>
       </c>
       <c r="C14" s="33">
         <f>'3 Unit economics'!C29</f>
@@ -8364,7 +8474,7 @@
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B18" s="11" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="C18" s="13">
         <f>(C6+C7)/2</f>
@@ -8373,43 +8483,43 @@
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B19" s="11" t="s">
-        <v>315</v>
+        <v>325</v>
       </c>
       <c r="C19" s="13">
         <f>(C7-C6)/2.5631</f>
         <v>312.12203971752956</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>316</v>
+        <v>326</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B20" s="11" t="s">
-        <v>317</v>
+        <v>327</v>
       </c>
       <c r="C20" s="27">
         <f>C15+C9-C8</f>
         <v>8.9293999999999993</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>318</v>
+        <v>328</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B21" s="5" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
       <c r="C21" s="18">
         <f>IFERROR(C14/(C14+C20),"")</f>
         <v>0.69491923287561119</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>320</v>
+        <v>330</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B22" s="11" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
       <c r="C22" s="13">
         <f>IFERROR(ROUND(NORMINV(C21,C18,C19),0),"")</f>
@@ -8418,7 +8528,7 @@
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B23" s="11" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="C23" s="13">
         <f>IFERROR(INT(C11/C15),"")</f>
@@ -8427,19 +8537,19 @@
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B24" s="5" t="s">
-        <v>323</v>
+        <v>333</v>
       </c>
       <c r="C24" s="17">
         <f>IFERROR(MIN(MAX(C10,C22),C23),"")</f>
         <v>386</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>324</v>
+        <v>334</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B25" s="11" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
       <c r="C25" s="14">
         <f>IFERROR((C24-C18)/C19,"")</f>
@@ -8448,7 +8558,7 @@
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B26" s="11" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="C26" s="13">
         <f>IFERROR(ROUND(C19*(NORMDIST(C25,0,1,FALSE)-C25*(1-NORMSDIST(C25))),0),"")</f>
@@ -8457,7 +8567,7 @@
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B27" s="11" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="C27" s="13">
         <f>IFERROR(ROUND(C24-C18+C26,0),"")</f>
@@ -8466,7 +8576,7 @@
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B28" s="11" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="C28" s="13">
         <f>IFERROR(ROUND(C14*(C18-C26)-C20*C27,0),"")</f>
@@ -8487,29 +8597,29 @@
     </row>
     <row r="33" spans="2:5" ht="26" x14ac:dyDescent="0.2">
       <c r="B33" s="3" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B35" s="4" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="C35" s="4"/>
     </row>
     <row r="36" spans="2:5" ht="65" x14ac:dyDescent="0.2">
       <c r="B36" s="11" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="C36" s="12">
         <v>44</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B37" s="11" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="C37" s="22">
         <v>12</v>
@@ -8517,7 +8627,7 @@
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B38" s="11" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
       <c r="C38" s="26">
         <v>0.04</v>
@@ -8525,7 +8635,7 @@
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B39" s="11" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="C39" s="26">
         <v>0.15</v>
@@ -8533,7 +8643,7 @@
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B40" s="11" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="C40" s="13">
         <f>IFERROR(ROUND(C36*(52/12)*C38*C37,0),"")</f>
@@ -8542,7 +8652,7 @@
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B41" s="11" t="s">
-        <v>337</v>
+        <v>347</v>
       </c>
       <c r="C41" s="13">
         <f>IFERROR(ROUND(C36*(52/12)*C39*C37,0),"")</f>
@@ -8551,7 +8661,7 @@
     </row>
     <row r="43" spans="2:5" ht="39" x14ac:dyDescent="0.2">
       <c r="B43" s="3" t="s">
-        <v>338</v>
+        <v>348</v>
       </c>
     </row>
   </sheetData>
@@ -8588,34 +8698,34 @@
     </row>
     <row r="2" spans="2:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>339</v>
+        <v>349</v>
       </c>
     </row>
     <row r="3" spans="2:10" ht="42" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>340</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B5" s="4" t="s">
-        <v>341</v>
+        <v>351</v>
       </c>
       <c r="C5" s="4"/>
       <c r="I5" s="4" t="s">
-        <v>342</v>
+        <v>352</v>
       </c>
       <c r="J5" s="4"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B6" s="11" t="s">
-        <v>343</v>
+        <v>353</v>
       </c>
       <c r="C6" s="33">
         <f>'3 Unit economics'!C6</f>
         <v>59.99</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>344</v>
+        <v>354</v>
       </c>
       <c r="J6" s="22">
         <v>39</v>
@@ -8630,7 +8740,7 @@
         <v>20.339570588235301</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>345</v>
+        <v>355</v>
       </c>
       <c r="J7" s="25">
         <v>3</v>
@@ -8638,14 +8748,14 @@
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B8" s="11" t="s">
-        <v>346</v>
+        <v>356</v>
       </c>
       <c r="C8" s="18">
         <f>IFERROR(C7/C6,"")</f>
         <v>0.3390493513624821</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>347</v>
+        <v>357</v>
       </c>
       <c r="J8" s="27">
         <f>IFERROR(J6*('6 Order size'!C15+J7),"")</f>
@@ -8654,14 +8764,14 @@
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B9" s="11" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
       <c r="C9" s="14">
         <f>IFERROR(1/C8,"")</f>
         <v>2.9494231325954874</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>349</v>
+        <v>359</v>
       </c>
       <c r="J9" s="27">
         <f>IFERROR(C18*8,"")</f>
@@ -8670,16 +8780,16 @@
     </row>
     <row r="10" spans="2:10" ht="65" x14ac:dyDescent="0.2">
       <c r="B10" s="11" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="C10" s="26">
         <v>0.3</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>351</v>
+        <v>361</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>352</v>
+        <v>362</v>
       </c>
       <c r="J10" s="28">
         <f>IFERROR(J8+J9,"")</f>
@@ -8688,7 +8798,7 @@
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B11" s="5" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
       <c r="C11" s="18">
         <f>IFERROR(C8*C10,"")</f>
@@ -8697,25 +8807,25 @@
     </row>
     <row r="12" spans="2:10" ht="65" x14ac:dyDescent="0.2">
       <c r="B12" s="11" t="s">
-        <v>354</v>
+        <v>364</v>
       </c>
       <c r="C12" s="14">
         <f>IFERROR(1/C11,"")</f>
         <v>9.8314104419849571</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B14" s="4" t="s">
-        <v>356</v>
+        <v>366</v>
       </c>
       <c r="C14" s="4"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B15" s="11" t="s">
-        <v>357</v>
+        <v>367</v>
       </c>
       <c r="C15" s="22">
         <v>3</v>
@@ -8723,7 +8833,7 @@
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
-        <v>358</v>
+        <v>368</v>
       </c>
       <c r="C16" s="25">
         <v>0.8</v>
@@ -8731,18 +8841,18 @@
     </row>
     <row r="17" spans="2:7" ht="117" x14ac:dyDescent="0.2">
       <c r="B17" s="11" t="s">
-        <v>359</v>
+        <v>369</v>
       </c>
       <c r="C17" s="26">
         <v>0.1</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="11" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="C18" s="27">
         <f>IFERROR(C15*C16/C17,"")</f>
@@ -8751,7 +8861,7 @@
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19" s="11" t="s">
-        <v>362</v>
+        <v>372</v>
       </c>
       <c r="C19" s="22">
         <v>4</v>
@@ -8759,7 +8869,7 @@
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="5" t="s">
-        <v>363</v>
+        <v>373</v>
       </c>
       <c r="C20" s="28">
         <f>IFERROR(C18*7*C19,"")</f>
@@ -8768,18 +8878,18 @@
     </row>
     <row r="21" spans="2:7" ht="39" x14ac:dyDescent="0.2">
       <c r="B21" s="3" t="s">
-        <v>364</v>
+        <v>374</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22" s="4" t="s">
-        <v>365</v>
+        <v>375</v>
       </c>
       <c r="C22" s="4"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="11" t="s">
-        <v>366</v>
+        <v>376</v>
       </c>
       <c r="C23" s="22">
         <v>15</v>
@@ -8787,7 +8897,7 @@
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="11" t="s">
-        <v>367</v>
+        <v>377</v>
       </c>
       <c r="C24" s="25">
         <v>10</v>
@@ -8795,7 +8905,7 @@
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25" s="5" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="C25" s="28">
         <f>IFERROR(SUMIFS($D$30:$D$229,$E$30:$E$229,0,$B$30:$B$229,"&lt;&gt;"),0)</f>
@@ -8804,7 +8914,7 @@
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="5" t="s">
-        <v>369</v>
+        <v>379</v>
       </c>
       <c r="C26" s="23">
         <f>COUNTIF($G$30:$G$229,"ADD AS NEGATIVE")</f>
@@ -8813,24 +8923,24 @@
     </row>
     <row r="28" spans="2:7" ht="39" x14ac:dyDescent="0.2">
       <c r="B28" s="3" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29" s="4" t="s">
-        <v>371</v>
+        <v>381</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>372</v>
+        <v>382</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>374</v>
+        <v>384</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>375</v>
+        <v>385</v>
       </c>
       <c r="G29" s="4" t="s">
         <v>75</v>
@@ -8838,7 +8948,7 @@
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="9" t="s">
-        <v>376</v>
+        <v>386</v>
       </c>
       <c r="C30" s="22">
         <v>42</v>
@@ -8859,7 +8969,7 @@
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" s="9" t="s">
-        <v>377</v>
+        <v>387</v>
       </c>
       <c r="C31" s="22">
         <v>23</v>
@@ -8880,7 +8990,7 @@
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="9" t="s">
-        <v>378</v>
+        <v>388</v>
       </c>
       <c r="C32" s="22">
         <v>35</v>

</xml_diff>